<commit_message>
added features in UI to better understaing and delay
</commit_message>
<xml_diff>
--- a/esempioTestFinale.xlsx
+++ b/esempioTestFinale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dev/Desktop/busplan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D866C6E-EEC1-E949-842A-62B7C6DF1484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37670C69-AB06-1541-A1D9-EC54BF0502D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5660" yWindow="500" windowWidth="23140" windowHeight="15880" xr2:uid="{738E9E6D-36A1-A142-ABA0-5C4E8C04C295}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
   <si>
     <t>Nome</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>Piazza Gavazzi, 1, 38057 Pergine Valsugana TN</t>
+  </si>
+  <si>
+    <t>IS Rovereto 2</t>
   </si>
 </sst>
 </file>
@@ -715,7 +718,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>28</v>

</xml_diff>